<commit_message>
Carga de datos: ubicacion por pasillo/rack/nivel, tipos automaticos, inspecciones; rubro en formulario publico; libros Codelco completos
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BD/Carga masiva/Presentacion/Codelco/2b_Activos_con_errores_para_mostrar.xlsx
+++ b/BD/Carga masiva/Presentacion/Codelco/2b_Activos_con_errores_para_mostrar.xlsx
@@ -2,6 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
@@ -22,50 +23,32 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="dd-mm-yyyy"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="dd-mm-yyyy"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
       <sz val="11"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="FF6732F4"/>
+      <color rgb="006732F4"/>
       <sz val="16"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <color rgb="FF68738A"/>
-      <sz val="11"/>
+      <b val="1"/>
+      <color rgb="0017223B"/>
     </font>
     <font>
-      <name val="Calibri"/>
       <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="FF17223B"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="FF68738A"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
+      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -74,21 +57,16 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2EFFF"/>
+        <fgColor rgb="00EAF4FF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEAF4FF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF6732F4"/>
+        <fgColor rgb="006732F4"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -96,43 +74,26 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FFE2E7F0"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -212,77 +173,82 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Vacío: se numera solo (ACT-&lt;n&gt;). Si lo escribe, queda ACT-&lt;lo escrito&gt;. No se cambia después: va en la etiqueta.</t>
+        <t>Opcional. Vacío: se numera solo (ACT-&lt;n&gt;). Si lo escribe, queda ACT-&lt;lo escrito&gt;. No se cambia después: va en la etiqueta. Ejemplo: EJEMPLO-HORNO-01</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>OBLIGATORIA. Cómo lo reconoce la gente.</t>
+        <t>Obligatoria. Cómo lo reconoce la gente. Ejemplo: Horno túnel línea 1</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>OBLIGATORIA. Tal como aparece en la hoja PLANTAS. Vea la hoja PLANTAS.</t>
+        <t>Obligatoria. Tal como aparece en la hoja PLANTAS. Ejemplo: Planta Renca</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Área de esa planta, como en la hoja AREAS. Vea la hoja AREAS.</t>
+        <t>Opcional. Área de esa planta, como en la hoja AREAS. Ejemplo: Producción</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>OBLIGATORIA. Como en la hoja TIPOS ACTIVO. Si no existe, se crea. Vea la hoja TIPOS ACTIVO.</t>
+        <t>Obligatoria. Como en la hoja TIPOS ACTIVO. Si no existe, se crea. Ejemplo: Horno</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>Si no existe para ese tipo, se crea.</t>
+        <t>Opcional. Si no existe para ese tipo, se crea. Ejemplo: HT-2000</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
-        <t>El fabricante.</t>
+        <t>Opcional. El fabricante. Ejemplo: Siemens</t>
       </text>
     </comment>
     <comment ref="H1" authorId="0" shapeId="0">
       <text>
-        <t>Número de serie de la placa.</t>
+        <t>Opcional. Número de serie de la placa. Ejemplo: SN-88231</t>
       </text>
     </comment>
     <comment ref="I1" authorId="0" shapeId="0">
       <text>
-        <t>OBLIGATORIA. Como en la hoja ESTADOS. Vea la hoja ESTADOS.</t>
+        <t>Obligatoria. Como en la hoja ESTADOS. Ejemplo: Operativo</t>
       </text>
     </comment>
     <comment ref="J1" authorId="0" shapeId="0">
       <text>
-        <t>OBLIGATORIA. Baja, Media, Alta o Crítica. Vea la hoja CRITICIDADES.</t>
+        <t>Obligatoria. Baja, Media, Alta o Crítica. Ejemplo: Alta</t>
       </text>
     </comment>
     <comment ref="K1" authorId="0" shapeId="0">
       <text>
-        <t>Como en la hoja CENTROS COSTO. Vea la hoja CENTROS COSTO.</t>
+        <t>Opcional. Como en la hoja CENTROS COSTO.</t>
       </text>
     </comment>
     <comment ref="L1" authorId="0" shapeId="0">
       <text>
-        <t>Código o nombre del activo principal (de la base o de esta hoja). Vacío: es una máquina principal.</t>
+        <t>Opcional. Código o nombre del activo principal (de la base o de esta hoja). Vacío: es una máquina principal.</t>
       </text>
     </comment>
     <comment ref="M1" authorId="0" shapeId="0">
       <text>
-        <t>Año, por ejemplo 2019.</t>
+        <t>Opcional. Año, por ejemplo 2019. Ejemplo: 2019</t>
       </text>
     </comment>
     <comment ref="N1" authorId="0" shapeId="0">
       <text>
-        <t>Fecha dd-mm-aaaa. No puede ser futura.</t>
+        <t>Opcional. Fecha dd-mm-aaaa. No puede ser futura.</t>
       </text>
     </comment>
     <comment ref="O1" authorId="0" shapeId="0">
       <text>
-        <t>NO lo deja deshabilitado. Vacío: SI. Valores: SI, NO.</t>
+        <t>Opcional. NO lo deja deshabilitado. Vacío: SI. Ejemplo: SI</t>
+      </text>
+    </comment>
+    <comment ref="P1" authorId="0" shapeId="0">
+      <text>
+        <t>Opcional.  Ejemplo: Horno a gas de 3 zonas</t>
       </text>
     </comment>
   </commentList>
@@ -297,22 +263,22 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>OBLIGATORIA. Código o nombre del activo (de la base o de la hoja ACTIVOS).</t>
+        <t>Obligatoria. Código o nombre del activo (de la base o de la hoja ACTIVOS). Ejemplo: EJEMPLO-HORNO-01</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>OBLIGATORIA. Qué característica: Potencia, Voltaje, Capacidad…</t>
+        <t>Obligatoria. Qué característica: Potencia, Voltaje, Capacidad… Ejemplo: Potencia</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>OBLIGATORIA. El valor tal como está en la placa o el manual.</t>
+        <t>Obligatoria. El valor tal como está en la placa o el manual. Ejemplo: 75</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Como en la hoja UNIDADES. Vea la hoja UNIDADES.</t>
+        <t>Opcional. Como en la hoja UNIDADES. Ejemplo: KW</t>
       </text>
     </comment>
   </commentList>
@@ -327,32 +293,37 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>OBLIGATORIA. Código o nombre del activo.</t>
+        <t>Obligatoria. Código o nombre del activo. Ejemplo: EJEMPLO-HORNO-01</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>OBLIGATORIA. Cómo se le dice a esa pieza.</t>
+        <t>Obligatoria. Cómo se le dice a esa pieza. Ejemplo: Motor ventilador</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Como en la hoja TIPOS COMPONENTE. Si no existe, se crea. Vacío: Otro. Vea la hoja TIPOS COMPONENTE.</t>
+        <t>Opcional. Como en la hoja TIPOS COMPONENTE. Si no existe, se crea. Vacío: Otro. Ejemplo: Motor</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Como en la hoja POSICIONES. Si no existe, se crea. Vea la hoja POSICIONES.</t>
+        <t>Opcional. Como en la hoja POSICIONES. Si no existe, se crea. Ejemplo: Lado accionamiento</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>Vacío: la del activo. Vea la hoja CRITICIDADES.</t>
+        <t>Opcional. Vacío: la del activo.</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>Vacío: hoy.</t>
+        <t>Opcional. Vacío: hoy.</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t xml:space="preserve">Opcional. </t>
       </text>
     </comment>
   </commentList>
@@ -367,47 +338,47 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>OBLIGATORIA. Código o nombre del activo.</t>
+        <t>Obligatoria. Código o nombre del activo. Ejemplo: EJEMPLO-HORNO-01</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Si se mide en una pieza: su nombre (de la base o de la hoja COMPONENTES).</t>
+        <t>Opcional. Si se mide en una pieza: su nombre (de la base o de la hoja COMPONENTES).</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>OBLIGATORIA. Qué se mide. Si no existe, se crea.</t>
+        <t>Obligatoria. Qué se mide. Si no existe, se crea. Ejemplo: Temperatura</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>OBLIGATORIA. Como en la hoja UNIDADES. Vea la hoja UNIDADES.</t>
+        <t>Obligatoria. Como en la hoja UNIDADES. Ejemplo: °C</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>Debajo de esto, SIGMA avisa.</t>
+        <t>Opcional. Debajo de esto, SIGMA avisa. Ejemplo: 180</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>Encima de esto, SIGMA avisa.</t>
+        <t>Opcional. Encima de esto, SIGMA avisa. Ejemplo: 240</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
-        <t>Valor de advertencia.</t>
+        <t>Opcional. Valor de advertencia.</t>
       </text>
     </comment>
     <comment ref="H1" authorId="0" shapeId="0">
       <text>
-        <t>Valor crítico.</t>
+        <t>Opcional. Valor crítico.</t>
       </text>
     </comment>
     <comment ref="I1" authorId="0" shapeId="0">
       <text>
-        <t>Cada cuántas horas se espera una lectura.</t>
+        <t>Opcional. Cada cuántas horas se espera una lectura.</t>
       </text>
     </comment>
   </commentList>
@@ -422,32 +393,32 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>OBLIGATORIA. Código o nombre del activo.</t>
+        <t>Obligatoria. Código o nombre del activo. Ejemplo: EJEMPLO-HORNO-01</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>OBLIGATORIA. Horómetro, Contador de ciclos, Odómetro…</t>
+        <t>Obligatoria. Horómetro, Contador de ciclos, Odómetro… Ejemplo: Horómetro</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>OBLIGATORIA. Como en la hoja UNIDADES (HORA, CICLO, KM…). Vea la hoja UNIDADES.</t>
+        <t>Obligatoria. Como en la hoja UNIDADES (HORA, CICLO, KM…). Ejemplo: HORA</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Lo que marca hoy. Vacío: 0.</t>
+        <t>Opcional. Lo que marca hoy. Vacío: 0. Ejemplo: 12500</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>SI si el contador puede volver a cero. Valores: SI, NO.</t>
+        <t>Opcional. SI si el contador puede volver a cero. Ejemplo: NO</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>Desde qué valor parte al reiniciar.</t>
+        <t>Opcional. Desde qué valor parte al reiniciar.</t>
       </text>
     </comment>
   </commentList>
@@ -462,17 +433,22 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>OBLIGATORIA. Código o nombre del activo.</t>
+        <t>Obligatoria. Código o nombre del activo. Ejemplo: EJEMPLO-HORNO-01</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Si es para una pieza: su nombre.</t>
+        <t>Opcional. Si es para una pieza: su nombre.</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>OBLIGATORIA. Código o nombre del repuesto, como en la hoja REPUESTOS. Vea la hoja REPUESTOS.</t>
+        <t>Obligatoria. Código o nombre del repuesto, como en la hoja REPUESTOS. Ejemplo: ROD-6205</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t xml:space="preserve">Opcional. </t>
       </text>
     </comment>
   </commentList>
@@ -768,7 +744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="150" customWidth="1" min="1" max="1"/>
@@ -782,115 +758,60 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Equipos y su jerarquía, datos técnicos, componentes, variables, medidores y los repuestos compatibles con cada uno. · Archivo con errores a propósito, solo para mostrar la revisión; no se carga.</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Equipos con su jerarquía, datos técnicos, componentes, variables, medidores y repuestos compatibles. · Archivo con errores a propósito, solo para mostrar la revisión; no se carga.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>1. Complete las hojas en el orden en que aparecen: cada una puede nombrar lo que crea una hoja anterior de este mismo archivo.</t>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1. Una hoja por paso, en el orden en que aparecen. Los encabezados MORADOS son obligatorios; los celestes, opcionales.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>2. Las columnas con encabezado MORADO son obligatorias para un registro nuevo; las celestes son opcionales.</t>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2. Pase el mouse por cada encabezado para ver qué escribir.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>3. Pase el mouse por cada encabezado para ver qué escribir. Las listas desplegables y las hojas de ayuda (al final) muestran los valores válidos.</t>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>3. Con el mismo código se ACTUALIZA: las celdas vacías conservan lo que había. Volver a cargar no duplica.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>4. La fila que empieza con EJEMPLO se ignora: bórrela o déjela.</t>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>4. Primero REVISE (no escribe nada) y después CARGUE. Una fila con error no detiene la carga.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>5. Con el mismo código se ACTUALIZA: las celdas con dato reemplazan y las vacías conservan lo que había. Volver a cargar el archivo no duplica.</t>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>5. La planta y las áreas (columna AREA = código del área) tienen que existir: se crean en Cliente › Organización.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>6. Primero REVISE: SIGMA dice qué pasará con cada fila (crear, actualizar, error) sin escribir nada. Después cargue.</t>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   El TIPO de activo, el modelo y la marca se crean si no existen.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>7. Una fila con error no detiene la carga: se informa con su hoja, fila, columna y motivo, y se descarga en Excel para corregir.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>HOJAS</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>ACTIVOS — Una fila por equipo, como los pasos 1 y 2 de la ficha. Con el mismo código (o el mismo nombre en la planta, si no lleva código) se actualiza.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>DATOS TECNICOS — Paso 3 de la ficha: una fila por dato (potencia, voltaje, capacidad…). Si el activo ya tenía ese dato, se reemplaza.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>COMPONENTES — Paso 4: las piezas que importan de cada equipo. Con el mismo nombre en el mismo activo se omite (no se duplica).</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>VARIABLES — Paso 5: lo que se mide para saber cómo está (temperatura, presión, vibración) y su rango normal. Si ya existe en ese activo, se omite.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>MEDIDORES — Paso 6: cuánto ha trabajado (horas, ciclos, km), con la lectura de hoy. Si ya existe en ese activo, se omite.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>REPUESTOS COMPATIBLES — Los repuestos de bodega que le sirven a cada equipo o componente. El repuesto tiene que existir (carga de Inventario). Si ya está vinculado, se omite.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="n"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Cargue antes el libro de Inventario: la hoja REPUESTOS COMPATIBLES nombra repuestos por su código.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -900,224 +821,222 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="FF6732F4"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:P7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" style="8" min="1" max="1"/>
-    <col width="30" customWidth="1" style="8" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" style="8" min="6" max="6"/>
-    <col width="16" customWidth="1" style="8" min="7" max="7"/>
-    <col width="16" customWidth="1" style="8" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" style="8" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" style="13" min="14" max="14"/>
-    <col width="9" customWidth="1" min="15" max="15"/>
-    <col width="34" customWidth="1" style="8" min="16" max="16"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="19" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="9" t="inlineStr">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>CODIGO</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>NOMBRE</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>PLANTA</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>AREA</t>
         </is>
       </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>TIPO</t>
         </is>
       </c>
-      <c r="F1" s="9" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>MODELO</t>
         </is>
       </c>
-      <c r="G1" s="9" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>MARCA</t>
         </is>
       </c>
-      <c r="H1" s="9" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>N SERIE</t>
         </is>
       </c>
-      <c r="I1" s="11" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>ESTADO</t>
         </is>
       </c>
-      <c r="J1" s="11" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>CRITICIDAD</t>
         </is>
       </c>
-      <c r="K1" s="6" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>CENTRO COSTO</t>
         </is>
       </c>
-      <c r="L1" s="9" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>DEPENDE DE</t>
         </is>
       </c>
-      <c r="M1" s="6" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>ANIO FABRICACION</t>
         </is>
       </c>
-      <c r="N1" s="14" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>PUESTA EN MARCHA</t>
         </is>
       </c>
-      <c r="O1" s="6" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>EN USO</t>
         </is>
       </c>
-      <c r="P1" s="9" t="inlineStr">
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>DESCRIPCION</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>CA-DEMO-OK-01</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>Chancador secundario de prueba</t>
         </is>
       </c>
-      <c r="C2" s="10" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>Concentradora Cerro Alto</t>
         </is>
       </c>
-      <c r="D2" s="10" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>CHA</t>
         </is>
       </c>
-      <c r="E2" s="10" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>Chancador</t>
         </is>
       </c>
-      <c r="F2" s="10" t="n"/>
-      <c r="G2" s="10" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>Metso</t>
         </is>
       </c>
-      <c r="H2" s="10" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>SN-DM-0001</t>
         </is>
       </c>
-      <c r="I2" s="10" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>Operativo</t>
         </is>
       </c>
-      <c r="J2" s="10" t="inlineStr">
+      <c r="J2" s="4" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="M2" s="7" t="n">
+      <c r="M2" t="n">
         <v>2022</v>
       </c>
-      <c r="N2" s="13" t="n">
+      <c r="N2" s="5" t="n">
         <v>44691</v>
       </c>
-      <c r="O2" s="10" t="inlineStr">
+      <c r="O2" s="4" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="P2" s="10" t="inlineStr">
+      <c r="P2" s="4" t="inlineStr">
         <is>
           <t>Fila correcta</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>CA-DEMO-OK-02</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Correa de transferencia de prueba</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Concentradora Cerro Alto</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>CHA</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>Correa transportadora</t>
         </is>
       </c>
-      <c r="G3" s="8" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>Fenner Dunlop</t>
         </is>
       </c>
-      <c r="H3" s="8" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>SN-DM-0002</t>
         </is>
       </c>
-      <c r="I3" s="8" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>Operativo</t>
         </is>
       </c>
-      <c r="J3" s="8" t="inlineStr">
+      <c r="J3" s="4" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="L3" s="8" t="inlineStr">
+      <c r="L3" s="4" t="inlineStr">
         <is>
           <t>CA-DEMO-OK-01</t>
         </is>
@@ -1125,52 +1044,52 @@
       <c r="M3" t="n">
         <v>2022</v>
       </c>
-      <c r="N3" s="13" t="n">
+      <c r="N3" s="5" t="n">
         <v>44691</v>
       </c>
-      <c r="O3" s="8" t="inlineStr">
+      <c r="O3" s="4" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="P3" s="8" t="inlineStr">
+      <c r="P3" s="4" t="inlineStr">
         <is>
           <t>Fila correcta (depende de la anterior)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>CA-DEMO-ERR-01</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Molino de prueba</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Planta Los Bronces</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>MOL</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Molino</t>
         </is>
       </c>
-      <c r="I4" s="8" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Operativo</t>
         </is>
       </c>
-      <c r="J4" s="8" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
@@ -1178,52 +1097,52 @@
       <c r="M4" t="n">
         <v>2021</v>
       </c>
-      <c r="N4" s="13" t="n">
+      <c r="N4" s="5" t="n">
         <v>44206</v>
       </c>
-      <c r="O4" s="8" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="P4" s="8" t="inlineStr">
+      <c r="P4" s="4" t="inlineStr">
         <is>
           <t>Error: la planta no existe</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>CA-DEMO-ERR-02</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Bomba de prueba</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Concentradora Cerro Alto</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>MOL</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Bomba de pulpa</t>
         </is>
       </c>
-      <c r="I5" s="8" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>Operativo</t>
         </is>
       </c>
-      <c r="J5" s="8" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>Extrema</t>
         </is>
@@ -1231,57 +1150,57 @@
       <c r="M5" t="n">
         <v>2021</v>
       </c>
-      <c r="N5" s="13" t="n">
+      <c r="N5" s="5" t="n">
         <v>44206</v>
       </c>
-      <c r="O5" s="8" t="inlineStr">
+      <c r="O5" s="4" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="P5" s="8" t="inlineStr">
+      <c r="P5" s="4" t="inlineStr">
         <is>
           <t>Error: la criticidad no existe</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>CA-DEMO-ERR-03</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Espesador de prueba</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Concentradora Cerro Alto</t>
         </is>
       </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>REL</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>Espesador</t>
         </is>
       </c>
-      <c r="I6" s="8" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>Operativo</t>
         </is>
       </c>
-      <c r="J6" s="8" t="inlineStr">
+      <c r="J6" s="4" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="L6" s="8" t="inlineStr">
+      <c r="L6" s="4" t="inlineStr">
         <is>
           <t>CA-NO-EXISTE</t>
         </is>
@@ -1289,63 +1208,58 @@
       <c r="M6" t="n">
         <v>2090</v>
       </c>
-      <c r="N6" s="13" t="n">
+      <c r="N6" s="5" t="n">
         <v>69399</v>
       </c>
-      <c r="O6" s="8" t="inlineStr">
+      <c r="O6" s="4" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="P6" s="8" t="inlineStr">
+      <c r="P6" s="4" t="inlineStr">
         <is>
           <t>Error: año y fecha futuros, y el activo padre no existe</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Celda de prueba</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Concentradora Cerro Alto</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>FLO</t>
         </is>
       </c>
-      <c r="I7" s="8" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>Operativo</t>
         </is>
       </c>
-      <c r="J7" s="8" t="inlineStr">
+      <c r="J7" s="4" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="O7" s="8" t="inlineStr">
+      <c r="O7" s="4" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="P7" s="8" t="inlineStr">
+      <c r="P7" s="4" t="inlineStr">
         <is>
           <t>Error: falta el tipo de activo</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="O2:O100000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"SI,NO"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
@@ -1354,80 +1268,79 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="FF6732F4"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" style="8" min="1" max="1"/>
-    <col width="20" customWidth="1" style="8" min="2" max="2"/>
-    <col width="14" customWidth="1" style="8" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>DATO</t>
         </is>
       </c>
-      <c r="C1" s="12" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>VALOR</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>UNIDAD</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>CA-DEMO-OK-01</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>Potencia</t>
         </is>
       </c>
-      <c r="C2" s="10" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>400</t>
         </is>
       </c>
-      <c r="D2" s="10" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>KW</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>CA-DEMO-ERR-02</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Potencia</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>150</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>KW</t>
         </is>
@@ -1442,81 +1355,80 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="FF6732F4"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" style="8" min="1" max="1"/>
-    <col width="26" customWidth="1" style="8" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" style="13" min="6" max="6"/>
-    <col width="30" customWidth="1" style="8" min="7" max="7"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>NOMBRE</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>QUE ES</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>DONDE VA</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>CRITICIDAD</t>
         </is>
       </c>
-      <c r="F1" s="14" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>FECHA INSTALACION</t>
         </is>
       </c>
-      <c r="G1" s="9" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>DESCRIPCION</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>CA-DEMO-OK-01</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>Motor principal</t>
         </is>
       </c>
-      <c r="C2" s="10" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>Motor</t>
         </is>
       </c>
-      <c r="D2" s="10" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Único</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
@@ -1531,77 +1443,69 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="FF6732F4"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" style="8" min="1" max="1"/>
-    <col width="20" customWidth="1" style="8" min="2" max="2"/>
-    <col width="18" customWidth="1" style="8" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="B1" s="9" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>COMPONENTE</t>
         </is>
       </c>
-      <c r="C1" s="12" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>VARIABLE</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>UNIDAD</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>MINIMO</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>MAXIMO</t>
         </is>
       </c>
-      <c r="G1" s="6" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>ADVERTENCIA</t>
         </is>
       </c>
-      <c r="H1" s="6" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>CRITICO</t>
         </is>
       </c>
-      <c r="I1" s="6" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>FRECUENCIA HORAS</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="10" t="n"/>
-      <c r="C2" s="10" t="n"/>
-      <c r="D2" s="7" t="n"/>
-      <c r="E2" s="7" t="n"/>
-      <c r="F2" s="7" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1612,84 +1516,78 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="FF6732F4"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" style="8" min="1" max="1"/>
-    <col width="20" customWidth="1" style="8" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>NOMBRE</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>UNIDAD</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>LECTURA ACTUAL</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>PERMITE REINICIO</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>VALOR REINICIO</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>CA-DEMO-OK-01</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>Horómetro</t>
         </is>
       </c>
-      <c r="C2" s="10" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>HORA</t>
         </is>
       </c>
-      <c r="D2" s="7" t="n">
+      <c r="D2" t="n">
         <v>100</v>
       </c>
-      <c r="E2" s="10" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="E2:E100000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"SI,NO"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
@@ -1698,44 +1596,39 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="FF6732F4"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" style="8" min="1" max="1"/>
-    <col width="20" customWidth="1" style="8" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" style="8" min="4" max="4"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>ACTIVO</t>
         </is>
       </c>
-      <c r="B1" s="9" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>COMPONENTE</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>REPUESTO</t>
         </is>
       </c>
-      <c r="D1" s="9" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>OBSERVACION</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="10" t="n"/>
-      <c r="C2" s="7" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>